<commit_message>
feat: BI vs. UB disambiguation framework + Fornell-Larcker extraction guidance + column cleanup
- Add BI vs. UB item-level linguistic decision framework (construct_harmonization.md Example 7)
- Expand BI/UB mapping rules with canonical reference items (Venkatesh 2003, Davis 1989, Thompson 1991)
- Add Fornell-Larcker CB-SEM vs. PLS-SEM extraction distinction with r_source flags
- Remove n_constructs_measured, n_correlations_reported, matrix_completeness from all XLSX
- Update coding manual to v2.3 with Section 7.6 disambiguation procedure
- Update codebook v1.1.0 with fornell_larcker_cbsem/plssem data_source values

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/AI_Adoption_MASEM_Coding_v1.xlsx
+++ b/data/templates/AI_Adoption_MASEM_Coding_v1.xlsx
@@ -2490,7 +2490,6 @@
           <t>float</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
           <t>Original beta if r was converted from beta</t>
@@ -2501,7 +2500,6 @@
           <t>0.38</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2571,7 +2569,6 @@
           <t>384</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2589,7 +2586,6 @@
           <t>string</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>Table/figure reference in the paper</t>
@@ -2600,7 +2596,6 @@
           <t>Table 3</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2618,7 +2613,6 @@
           <t>integer</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr">
         <is>
           <t>Page number in the paper</t>
@@ -2629,7 +2623,6 @@
           <t>12</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2647,7 +2640,6 @@
           <t>string</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr">
         <is>
           <t>Any notes about this correlation</t>
@@ -2658,7 +2650,6 @@
           <t>Bootstrapped CI reported</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3358,7 +3349,6 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4086,7 +4076,6 @@
           <t>integer</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr">
         <is>
           <t>Study identifier</t>
@@ -4097,7 +4086,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4115,7 +4103,6 @@
           <t>string</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr">
         <is>
           <t>Construct pair identifier</t>
@@ -4126,7 +4113,6 @@
           <t>PE-BI</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4144,7 +4130,6 @@
           <t>string</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr">
         <is>
           <t>Variable where discrepancy occurred</t>
@@ -4155,7 +4140,6 @@
           <t>r</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4173,7 +4157,6 @@
           <t>string</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr">
         <is>
           <t>Value from first coder</t>
@@ -4184,7 +4167,6 @@
           <t>0.45</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4202,7 +4184,6 @@
           <t>string</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
         <is>
           <t>Value from second coder</t>
@@ -4213,7 +4194,6 @@
           <t>0.43</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -4305,7 +4285,6 @@
           <t>string</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr">
         <is>
           <t>Resolved final value</t>
@@ -4316,7 +4295,6 @@
           <t>0.45</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4371,7 +4349,6 @@
           <t>string</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
         <is>
           <t>Who resolved the discrepancy</t>
@@ -4382,7 +4359,6 @@
           <t>HK</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5059,7 +5035,6 @@
           <t>string</t>
         </is>
       </c>
-      <c r="D135" t="inlineStr"/>
       <c r="E135" t="inlineStr">
         <is>
           <t>Full search query used</t>
@@ -5070,7 +5045,6 @@
           <t>("artificial intelligence" OR "AI") AND ("adoption" OR "acceptance")</t>
         </is>
       </c>
-      <c r="G135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5103,7 +5077,6 @@
           <t>1247</t>
         </is>
       </c>
-      <c r="G136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -5121,7 +5094,6 @@
           <t>string</t>
         </is>
       </c>
-      <c r="D137" t="inlineStr"/>
       <c r="E137" t="inlineStr">
         <is>
           <t>Notes about this search</t>
@@ -5132,7 +5104,6 @@
           <t>Limited to 2015-2025</t>
         </is>
       </c>
-      <c r="G137" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G137"/>
@@ -5147,7 +5118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY1"/>
+  <dimension ref="A1:AV1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5326,135 +5297,120 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>n_constructs_measured</t>
+          <t>measures_BI</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>measures_BI</t>
+          <t>measures_UB</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>measures_UB</t>
+          <t>adoption_dv_type</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>adoption_dv_type</t>
+          <t>reporting_quality</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>n_correlations_reported</t>
+          <t>sample_adequacy</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>matrix_completeness</t>
+          <t>construct_validity</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>reporting_quality</t>
+          <t>common_method_bias</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>sample_adequacy</t>
+          <t>overall_quality</t>
         </is>
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>construct_validity</t>
+          <t>rob_notes</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>common_method_bias</t>
+          <t>screen_decision_codex</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
-          <t>overall_quality</t>
+          <t>screen_decision_gemini</t>
         </is>
       </c>
       <c r="AJ1" s="1" t="inlineStr">
         <is>
-          <t>rob_notes</t>
+          <t>screen_consensus</t>
         </is>
       </c>
       <c r="AK1" s="1" t="inlineStr">
         <is>
-          <t>screen_decision_codex</t>
+          <t>human1_decision</t>
         </is>
       </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
-          <t>screen_decision_gemini</t>
+          <t>human2_decision</t>
         </is>
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
-          <t>screen_consensus</t>
+          <t>adjudicated_final_decision</t>
         </is>
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>human1_decision</t>
+          <t>exclude_code</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>human2_decision</t>
+          <t>decision_rationale</t>
         </is>
       </c>
       <c r="AP1" s="1" t="inlineStr">
         <is>
-          <t>adjudicated_final_decision</t>
+          <t>adjudicator_id</t>
         </is>
       </c>
       <c r="AQ1" s="1" t="inlineStr">
         <is>
-          <t>exclude_code</t>
+          <t>screen_run_id</t>
         </is>
       </c>
       <c r="AR1" s="1" t="inlineStr">
         <is>
-          <t>decision_rationale</t>
+          <t>oauth_auth_method_codex</t>
         </is>
       </c>
       <c r="AS1" s="1" t="inlineStr">
         <is>
-          <t>adjudicator_id</t>
+          <t>oauth_auth_method_gemini</t>
         </is>
       </c>
       <c r="AT1" s="1" t="inlineStr">
         <is>
-          <t>screen_run_id</t>
+          <t>human_coder</t>
         </is>
       </c>
       <c r="AU1" s="1" t="inlineStr">
         <is>
-          <t>oauth_auth_method_codex</t>
+          <t>coding_date</t>
         </is>
       </c>
       <c r="AV1" s="1" t="inlineStr">
-        <is>
-          <t>oauth_auth_method_gemini</t>
-        </is>
-      </c>
-      <c r="AW1" s="1" t="inlineStr">
-        <is>
-          <t>human_coder</t>
-        </is>
-      </c>
-      <c r="AX1" s="1" t="inlineStr">
-        <is>
-          <t>coding_date</t>
-        </is>
-      </c>
-      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>coding_notes</t>
         </is>

</xml_diff>